<commit_message>
refined simulations and results
</commit_message>
<xml_diff>
--- a/data/inventories_ei310.xlsx
+++ b/data/inventories_ei310.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anabera\Desktop\Side projects\Nitrous oxide production\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F0FEF68-E419-4A1F-94DF-4746AAC7B520}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40399F58-DCCB-4FE8-A2F6-77C835E753C5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="495" windowWidth="14400" windowHeight="4110" activeTab="3" xr2:uid="{79F87D26-5407-4579-9D8D-FA563FE5FD90}"/>
   </bookViews>
@@ -357,21 +357,9 @@
     <t>ammonia, anhydrous, liquid</t>
   </si>
   <si>
-    <t>nitrous oxide production, AON ideal, fossil ammonia</t>
-  </si>
-  <si>
-    <t>nitrous oxide production, AON ideal, green ammonia</t>
-  </si>
-  <si>
     <t>ecoinvent-3.10-cutoff-Base-2020</t>
   </si>
   <si>
-    <t>nitrous oxide production, AON real, fossil ammonia</t>
-  </si>
-  <si>
-    <t>nitrous oxide production, AON real, green ammonia</t>
-  </si>
-  <si>
     <t>Dinitrogen monoxide</t>
   </si>
   <si>
@@ -384,12 +372,6 @@
     <t xml:space="preserve">GLO </t>
   </si>
   <si>
-    <t>hydrogen peroxide production, AO real, fossil hydrogen</t>
-  </si>
-  <si>
-    <t>hydrogen peroxide production, AO real, green hydrogen</t>
-  </si>
-  <si>
     <t xml:space="preserve">anthraquinone </t>
   </si>
   <si>
@@ -409,6 +391,24 @@
   </si>
   <si>
     <t>benzene</t>
+  </si>
+  <si>
+    <t>nitrous oxide production, AON 88, fossil ammonia</t>
+  </si>
+  <si>
+    <t>nitrous oxide production, AON 100, fossil ammonia</t>
+  </si>
+  <si>
+    <t>hydrogen peroxide production, AO, green hydrogen</t>
+  </si>
+  <si>
+    <t>hydrogen peroxide production, AO, fossil hydrogen</t>
+  </si>
+  <si>
+    <t>nitrous oxide production, AON 100, green ammonia</t>
+  </si>
+  <si>
+    <t>nitrous oxide production, AON 88, green ammonia</t>
   </si>
 </sst>
 </file>
@@ -1092,7 +1092,7 @@
         <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
@@ -1115,7 +1115,7 @@
         <v>15</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
@@ -1138,7 +1138,7 @@
         <v>15</v>
       </c>
       <c r="G15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
@@ -1339,7 +1339,7 @@
         <v>3</v>
       </c>
       <c r="G27" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H27" t="s">
         <v>16</v>
@@ -1362,7 +1362,7 @@
         <v>15</v>
       </c>
       <c r="G28" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H28" t="s">
         <v>16</v>
@@ -1385,7 +1385,7 @@
         <v>3</v>
       </c>
       <c r="G29" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H29" t="s">
         <v>16</v>
@@ -1408,7 +1408,7 @@
         <v>15</v>
       </c>
       <c r="G30" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H30" t="s">
         <v>16</v>
@@ -1431,7 +1431,7 @@
         <v>15</v>
       </c>
       <c r="G31" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H31" t="s">
         <v>16</v>
@@ -1454,7 +1454,7 @@
         <v>15</v>
       </c>
       <c r="G32" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H32" t="s">
         <v>16</v>
@@ -1477,7 +1477,7 @@
         <v>15</v>
       </c>
       <c r="G33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H33" t="s">
         <v>16</v>
@@ -1500,7 +1500,7 @@
         <v>15</v>
       </c>
       <c r="G34" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H34" t="s">
         <v>16</v>
@@ -1523,7 +1523,7 @@
         <v>15</v>
       </c>
       <c r="G35" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H35" t="s">
         <v>16</v>
@@ -1546,7 +1546,7 @@
         <v>3</v>
       </c>
       <c r="G36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H36" t="s">
         <v>16</v>
@@ -1569,7 +1569,7 @@
         <v>15</v>
       </c>
       <c r="G37" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H37" t="s">
         <v>16</v>
@@ -1592,7 +1592,7 @@
         <v>15</v>
       </c>
       <c r="G38" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H38" t="s">
         <v>16</v>
@@ -1615,7 +1615,7 @@
         <v>15</v>
       </c>
       <c r="G39" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H39" t="s">
         <v>16</v>
@@ -1638,7 +1638,7 @@
         <v>15</v>
       </c>
       <c r="G40" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H40" t="s">
         <v>16</v>
@@ -1661,7 +1661,7 @@
         <v>15</v>
       </c>
       <c r="G41" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H41" t="s">
         <v>16</v>
@@ -1879,7 +1879,7 @@
         <v>15</v>
       </c>
       <c r="G54" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H54" t="s">
         <v>16</v>
@@ -1902,7 +1902,7 @@
         <v>15</v>
       </c>
       <c r="G55" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H55" t="s">
         <v>16</v>
@@ -1925,7 +1925,7 @@
         <v>15</v>
       </c>
       <c r="G56" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H56" t="s">
         <v>16</v>
@@ -1948,7 +1948,7 @@
         <v>15</v>
       </c>
       <c r="G57" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H57" t="s">
         <v>16</v>
@@ -1971,7 +1971,7 @@
         <v>15</v>
       </c>
       <c r="G58" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H58" t="s">
         <v>16</v>
@@ -1994,7 +1994,7 @@
         <v>15</v>
       </c>
       <c r="G59" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H59" t="s">
         <v>16</v>
@@ -2017,7 +2017,7 @@
         <v>15</v>
       </c>
       <c r="G60" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H60" t="s">
         <v>16</v>
@@ -2040,7 +2040,7 @@
         <v>15</v>
       </c>
       <c r="G61" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H61" t="s">
         <v>16</v>
@@ -2063,7 +2063,7 @@
         <v>15</v>
       </c>
       <c r="G62" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H62" t="s">
         <v>16</v>
@@ -2345,7 +2345,7 @@
         <v>3</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
@@ -2368,7 +2368,7 @@
         <v>3</v>
       </c>
       <c r="G15" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
@@ -2391,7 +2391,7 @@
         <v>15</v>
       </c>
       <c r="G16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H16" t="s">
         <v>16</v>
@@ -2695,7 +2695,7 @@
         <v>15</v>
       </c>
       <c r="G33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H33" t="s">
         <v>16</v>
@@ -2895,7 +2895,7 @@
         <v>3</v>
       </c>
       <c r="G45" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H45" t="s">
         <v>16</v>
@@ -2918,7 +2918,7 @@
         <v>15</v>
       </c>
       <c r="G46" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H46" t="s">
         <v>16</v>
@@ -2941,7 +2941,7 @@
         <v>15</v>
       </c>
       <c r="G47" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H47" t="s">
         <v>16</v>
@@ -2964,7 +2964,7 @@
         <v>3</v>
       </c>
       <c r="G48" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H48" t="s">
         <v>16</v>
@@ -3144,7 +3144,7 @@
         <v>3</v>
       </c>
       <c r="G59" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H59" t="s">
         <v>16</v>
@@ -3239,7 +3239,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C1" s="16"/>
       <c r="D1" s="3"/>
@@ -3293,7 +3293,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="3"/>
@@ -3356,10 +3356,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B9" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="C9" s="11">
         <v>1</v>
@@ -3394,7 +3394,7 @@
         <v>15</v>
       </c>
       <c r="G10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -3417,7 +3417,7 @@
         <v>15</v>
       </c>
       <c r="G11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
@@ -3440,7 +3440,7 @@
         <v>3</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -3484,7 +3484,7 @@
         <v>0</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="3"/>
@@ -3538,7 +3538,7 @@
         <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="3"/>
@@ -3601,10 +3601,10 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="B23" t="s">
-        <v>110</v>
+        <v>125</v>
       </c>
       <c r="C23" s="11">
         <v>1</v>
@@ -3662,7 +3662,7 @@
         <v>15</v>
       </c>
       <c r="G25" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H25" t="s">
         <v>16</v>
@@ -3685,7 +3685,7 @@
         <v>3</v>
       </c>
       <c r="G26" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H26" t="s">
         <v>16</v>
@@ -3729,7 +3729,7 @@
         <v>0</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="3"/>
@@ -3783,7 +3783,7 @@
         <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C33" s="16"/>
       <c r="D33" s="3"/>
@@ -3846,10 +3846,10 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="B37" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C37" s="11">
         <v>1</v>
@@ -3875,7 +3875,7 @@
         <v>107</v>
       </c>
       <c r="C38" s="11">
-        <v>0.96854616228089385</v>
+        <v>0.91964998512365381</v>
       </c>
       <c r="D38" t="s">
         <v>7</v>
@@ -3884,7 +3884,7 @@
         <v>15</v>
       </c>
       <c r="G38" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H38" t="s">
         <v>16</v>
@@ -3898,7 +3898,7 @@
         <v>88</v>
       </c>
       <c r="C39" s="12">
-        <v>-1.5899795617732801E-3</v>
+        <v>-1.51353683099332E-3</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
@@ -3907,7 +3907,7 @@
         <v>15</v>
       </c>
       <c r="G39" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H39" t="s">
         <v>16</v>
@@ -3921,7 +3921,7 @@
         <v>34</v>
       </c>
       <c r="C40" s="12">
-        <v>6.5803725096832189E-2</v>
+        <v>6.0754013722332099E-2</v>
       </c>
       <c r="D40" t="s">
         <v>35</v>
@@ -3930,7 +3930,7 @@
         <v>3</v>
       </c>
       <c r="G40" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H40" t="s">
         <v>16</v>
@@ -3944,7 +3944,7 @@
         <v>99</v>
       </c>
       <c r="C41" s="11">
-        <v>19.451798344592323</v>
+        <v>4.6646502651840436</v>
       </c>
       <c r="D41" t="s">
         <v>29</v>
@@ -3961,22 +3961,22 @@
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B42" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C42" s="11">
-        <v>0.57280190681669141</v>
+        <v>0.50722214107282404</v>
       </c>
       <c r="D42" t="s">
         <v>29</v>
       </c>
       <c r="E42" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G42" s="21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H42" t="s">
         <v>16</v>
@@ -3987,7 +3987,7 @@
         <v>101</v>
       </c>
       <c r="C43" s="12">
-        <v>8.5167437462212083E-3</v>
+        <v>7.842128857001375E-2</v>
       </c>
       <c r="D43" s="22" t="s">
         <v>7</v>
@@ -4004,10 +4004,10 @@
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B44" t="s">
-        <v>114</v>
-      </c>
-      <c r="C44" s="23">
-        <v>1.5175217048085957E-5</v>
+        <v>110</v>
+      </c>
+      <c r="C44" s="13">
+        <v>2.0022743606470884E-4</v>
       </c>
       <c r="D44" s="22" t="s">
         <v>7</v>
@@ -4027,7 +4027,7 @@
         <v>21</v>
       </c>
       <c r="C45" s="12">
-        <v>6.7533182458830068E-2</v>
+        <v>1.4556189599066783E-2</v>
       </c>
       <c r="D45" s="22" t="s">
         <v>7</v>
@@ -4057,7 +4057,7 @@
         <v>0</v>
       </c>
       <c r="B47" s="8" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C47" s="16"/>
       <c r="D47" s="3"/>
@@ -4111,7 +4111,7 @@
         <v>5</v>
       </c>
       <c r="B51" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C51" s="16"/>
       <c r="D51" s="3"/>
@@ -4174,10 +4174,10 @@
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="B55" t="s">
-        <v>113</v>
+        <v>126</v>
       </c>
       <c r="C55" s="11">
         <v>1</v>
@@ -4203,7 +4203,7 @@
         <v>106</v>
       </c>
       <c r="C56" s="11">
-        <v>0.96854616228089385</v>
+        <v>0.91964998512365381</v>
       </c>
       <c r="D56" t="s">
         <v>7</v>
@@ -4226,7 +4226,7 @@
         <v>88</v>
       </c>
       <c r="C57" s="12">
-        <v>-1.5899795617732801E-3</v>
+        <v>-1.51353683099332E-3</v>
       </c>
       <c r="D57" t="s">
         <v>17</v>
@@ -4235,7 +4235,7 @@
         <v>15</v>
       </c>
       <c r="G57" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H57" t="s">
         <v>16</v>
@@ -4249,7 +4249,7 @@
         <v>34</v>
       </c>
       <c r="C58" s="12">
-        <v>6.5803725096832189E-2</v>
+        <v>6.0754013722332099E-2</v>
       </c>
       <c r="D58" t="s">
         <v>35</v>
@@ -4258,7 +4258,7 @@
         <v>3</v>
       </c>
       <c r="G58" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H58" t="s">
         <v>16</v>
@@ -4272,7 +4272,7 @@
         <v>99</v>
       </c>
       <c r="C59" s="11">
-        <v>19.451798344592323</v>
+        <v>4.6646502651840436</v>
       </c>
       <c r="D59" t="s">
         <v>29</v>
@@ -4289,22 +4289,22 @@
     </row>
     <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B60" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="C60" s="11">
-        <v>0.57280190681669141</v>
+        <v>0.50722214107282404</v>
       </c>
       <c r="D60" t="s">
         <v>29</v>
       </c>
       <c r="E60" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G60" s="21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H60" t="s">
         <v>16</v>
@@ -4315,7 +4315,7 @@
         <v>101</v>
       </c>
       <c r="C61" s="12">
-        <v>8.5167437462212083E-3</v>
+        <v>7.842128857001375E-2</v>
       </c>
       <c r="D61" s="22" t="s">
         <v>7</v>
@@ -4332,10 +4332,10 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B62" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C62" s="23">
-        <v>1.5175217048085957E-5</v>
+        <v>2.0022743606470884E-4</v>
       </c>
       <c r="D62" s="22" t="s">
         <v>7</v>
@@ -4355,7 +4355,7 @@
         <v>21</v>
       </c>
       <c r="C63" s="12">
-        <v>6.7533182458830068E-2</v>
+        <v>1.4556189599066783E-2</v>
       </c>
       <c r="D63" s="22" t="s">
         <v>7</v>
@@ -4396,7 +4396,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C1" s="16"/>
       <c r="D1" s="3"/>
@@ -4450,7 +4450,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C5" s="16"/>
       <c r="D5" s="3"/>
@@ -4513,10 +4513,10 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="B9" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C9" s="11">
         <v>1</v>
@@ -4536,10 +4536,10 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B10" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C10" s="12">
         <v>6.5856585494280195E-2</v>
@@ -4551,7 +4551,7 @@
         <v>15</v>
       </c>
       <c r="G10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
@@ -4559,10 +4559,10 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B11" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C11" s="12">
         <v>3.0874916157909655E-3</v>
@@ -4574,7 +4574,7 @@
         <v>3</v>
       </c>
       <c r="G11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
@@ -4582,10 +4582,10 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B12" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C12" s="12">
         <v>1.9300000000000001E-3</v>
@@ -4597,7 +4597,7 @@
         <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
@@ -4620,7 +4620,7 @@
         <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
@@ -4643,7 +4643,7 @@
         <v>3</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H14" t="s">
         <v>16</v>
@@ -4689,7 +4689,7 @@
         <v>15</v>
       </c>
       <c r="G16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H16" t="s">
         <v>16</v>
@@ -4717,7 +4717,7 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B18" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C18" s="11">
         <f>2.9831*C11</f>
@@ -4772,7 +4772,7 @@
         <v>0</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C21" s="16"/>
       <c r="D21" s="3"/>
@@ -4826,7 +4826,7 @@
         <v>5</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="3"/>
@@ -4889,10 +4889,10 @@
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B29" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="C29" s="11">
         <v>1</v>
@@ -4935,10 +4935,10 @@
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="B31" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C31" s="12">
         <v>3.0874916157909655E-3</v>
@@ -4950,7 +4950,7 @@
         <v>3</v>
       </c>
       <c r="G31" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H31" t="s">
         <v>16</v>
@@ -4958,10 +4958,10 @@
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="B32" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C32" s="12">
         <v>1.9300000000000001E-3</v>
@@ -4973,7 +4973,7 @@
         <v>15</v>
       </c>
       <c r="G32" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H32" t="s">
         <v>16</v>
@@ -4996,7 +4996,7 @@
         <v>15</v>
       </c>
       <c r="G33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H33" t="s">
         <v>16</v>
@@ -5019,7 +5019,7 @@
         <v>3</v>
       </c>
       <c r="G34" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H34" t="s">
         <v>16</v>
@@ -5065,7 +5065,7 @@
         <v>15</v>
       </c>
       <c r="G36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H36" t="s">
         <v>16</v>
@@ -5093,7 +5093,7 @@
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C38" s="11">
         <f>2.9831*C31</f>

</xml_diff>